<commit_message>
Backup: Complete UI redesign, dual logos, smart Excel COM navigation, and custom expiration thresholds
</commit_message>
<xml_diff>
--- a/Copy of VehicleMonitoring.xlsx
+++ b/Copy of VehicleMonitoring.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" firstSheet="5" activeTab="9"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="APRIL 2024" sheetId="1" r:id="rId1"/>
@@ -20,17 +20,6 @@
     <sheet name="APRIL 2025" sheetId="11" r:id="rId11"/>
   </sheets>
   <calcPr calcId="145621"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
@@ -1516,6 +1505,9 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1524,9 +1516,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2116,9 +2105,6 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
     </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
   </extLst>
 </styleSheet>
 </file>
@@ -2138,7 +2124,7 @@
         <xdr:cNvPr id="2" name="TextBox 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2477,7 +2463,7 @@
     <row r="2" spans="1:16">
       <c r="A2" s="75">
         <f ca="1">TODAY()</f>
-        <v>46083</v>
+        <v>46085</v>
       </c>
     </row>
     <row r="3" spans="1:16">
@@ -2631,7 +2617,7 @@
         <v>45717</v>
       </c>
       <c r="K8" s="14" t="str">
-        <f t="shared" ref="K8:K9" ca="1" si="0">IF(A8="YES","REGISTERED",IF(J8="","PLEASE INPUT LAST REG",IF(J8-TODAY()&lt;0,"EXPIRED",IF(J8-TODAY()&lt;=14,J8-TODAY()&amp;" DAYS BEFORE EXPIRY",IF(AND(J8-TODAY()&gt;14,J8-TODAY()&lt;=29),J9-TODAY()&amp;" DAYS BEFORE 2 WEEK NOTICE",IF(J8-TODAY()&gt;=30,"Sufficient Time"))))))</f>
+        <f ca="1">IF(A8="YES","REGISTERED",IF(J8="","PLEASE INPUT LAST REG",IF(J8-TODAY()&lt;0,"EXPIRED",IF(J8-TODAY()&lt;=14,J8-TODAY()&amp;" DAYS BEFORE EXPIRY",IF(AND(J8-TODAY()&gt;14,J8-TODAY()&lt;=29),J9-TODAY()&amp;" DAYS BEFORE 2 WEEK NOTICE",IF(J8-TODAY()&gt;=30,"Sufficient Time"))))))</f>
         <v>EXPIRED</v>
       </c>
       <c r="L8" s="57" t="s">
@@ -2673,7 +2659,7 @@
         <v>45717</v>
       </c>
       <c r="K9" s="14" t="str">
-        <f t="shared" ca="1" si="0"/>
+        <f ca="1">IF(A9="YES","REGISTERED",IF(J9="","PLEASE INPUT LAST REG",IF(J9-TODAY()&lt;0,"EXPIRED",IF(J9-TODAY()&lt;=14,J9-TODAY()&amp;" DAYS BEFORE EXPIRY",IF(AND(J9-TODAY()&gt;14,J9-TODAY()&lt;=29),J10-TODAY()&amp;" DAYS BEFORE 2 WEEK NOTICE",IF(J9-TODAY()&gt;=30,"Sufficient Time"))))))</f>
         <v>EXPIRED</v>
       </c>
       <c r="L9" s="83" t="s">
@@ -2901,7 +2887,7 @@
     <row r="2" spans="1:16">
       <c r="A2" s="85">
         <f ca="1">TODAY()</f>
-        <v>46083</v>
+        <v>46085</v>
       </c>
     </row>
     <row r="4" spans="1:16">
@@ -3230,8 +3216,12 @@
         <v>9809.4699999999993</v>
       </c>
       <c r="H12" s="10"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
+      <c r="I12" s="31">
+        <v>45733</v>
+      </c>
+      <c r="J12" s="31">
+        <v>46068</v>
+      </c>
       <c r="K12" s="6" t="str">
         <f t="shared" ca="1" si="0"/>
         <v>REGISTERED</v>
@@ -3524,7 +3514,7 @@
     <row r="2" spans="1:16">
       <c r="A2" s="75">
         <f ca="1">TODAY()</f>
-        <v>46083</v>
+        <v>46085</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="14.45" customHeight="1">
@@ -3979,22 +3969,22 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="I6:I7"/>
-    <mergeCell ref="J6:J7"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="E6:E7"/>
     <mergeCell ref="N6:N7"/>
     <mergeCell ref="O6:O7"/>
     <mergeCell ref="P6:P7"/>
     <mergeCell ref="G4:L5"/>
     <mergeCell ref="L6:M6"/>
     <mergeCell ref="K6:K7"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="I6:I7"/>
+    <mergeCell ref="J6:J7"/>
   </mergeCells>
   <conditionalFormatting sqref="K8:K14">
     <cfRule type="containsText" dxfId="53" priority="1" operator="containsText" text="REGISTERED">
@@ -4057,7 +4047,7 @@
     <row r="2" spans="1:16">
       <c r="A2" s="18">
         <f ca="1">TODAY()</f>
-        <v>46083</v>
+        <v>46085</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="14.45" customHeight="1">
@@ -4718,11 +4708,6 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="E6:E7"/>
     <mergeCell ref="N6:N7"/>
     <mergeCell ref="O6:O7"/>
     <mergeCell ref="P6:P7"/>
@@ -4734,6 +4719,11 @@
     <mergeCell ref="I6:I7"/>
     <mergeCell ref="J6:J7"/>
     <mergeCell ref="K6:K7"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E6:E7"/>
   </mergeCells>
   <conditionalFormatting sqref="K8:K18">
     <cfRule type="containsText" dxfId="47" priority="1" operator="containsText" text="REGISTERED">
@@ -4793,7 +4783,7 @@
     <row r="2" spans="1:16">
       <c r="A2" s="18">
         <f ca="1">TODAY()</f>
-        <v>46083</v>
+        <v>46085</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="26.25">
@@ -5462,22 +5452,22 @@
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="H6:H7"/>
-    <mergeCell ref="I6:I7"/>
-    <mergeCell ref="J6:J7"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="B6:B7"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="D6:D7"/>
-    <mergeCell ref="E6:E7"/>
     <mergeCell ref="N6:N7"/>
     <mergeCell ref="O6:O7"/>
     <mergeCell ref="P6:P7"/>
     <mergeCell ref="G4:K5"/>
     <mergeCell ref="L6:M6"/>
     <mergeCell ref="K6:K7"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="B6:B7"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="D6:D7"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="H6:H7"/>
+    <mergeCell ref="I6:I7"/>
+    <mergeCell ref="J6:J7"/>
   </mergeCells>
   <conditionalFormatting sqref="K8:K20">
     <cfRule type="containsText" dxfId="41" priority="1" operator="containsText" text="REGISTERED">
@@ -5539,7 +5529,7 @@
     <row r="2" spans="1:16" ht="21" customHeight="1">
       <c r="A2" s="18">
         <f ca="1">TODAY()</f>
-        <v>46083</v>
+        <v>46085</v>
       </c>
       <c r="G2" s="98" t="s">
         <v>1</v>
@@ -5562,34 +5552,34 @@
       <c r="A4" s="93" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="104" t="s">
+      <c r="B4" s="101" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="104" t="s">
+      <c r="C4" s="101" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="104" t="s">
+      <c r="D4" s="101" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="104" t="s">
+      <c r="E4" s="101" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="104" t="s">
+      <c r="F4" s="101" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="104" t="s">
+      <c r="G4" s="101" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="101" t="s">
+      <c r="H4" s="102" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="101" t="s">
+      <c r="I4" s="102" t="s">
         <v>10</v>
       </c>
-      <c r="J4" s="101" t="s">
+      <c r="J4" s="102" t="s">
         <v>11</v>
       </c>
-      <c r="K4" s="101" t="s">
+      <c r="K4" s="102" t="s">
         <v>12</v>
       </c>
       <c r="L4" s="44" t="s">
@@ -5602,22 +5592,22 @@
       <c r="O4" s="43" t="s">
         <v>15</v>
       </c>
-      <c r="P4" s="103" t="s">
+      <c r="P4" s="104" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="5" spans="1:16">
       <c r="A5" s="100"/>
-      <c r="B5" s="104"/>
-      <c r="C5" s="104"/>
-      <c r="D5" s="104"/>
-      <c r="E5" s="104"/>
-      <c r="F5" s="104"/>
-      <c r="G5" s="104"/>
-      <c r="H5" s="102"/>
-      <c r="I5" s="102"/>
-      <c r="J5" s="102"/>
-      <c r="K5" s="102"/>
+      <c r="B5" s="101"/>
+      <c r="C5" s="101"/>
+      <c r="D5" s="101"/>
+      <c r="E5" s="101"/>
+      <c r="F5" s="101"/>
+      <c r="G5" s="101"/>
+      <c r="H5" s="103"/>
+      <c r="I5" s="103"/>
+      <c r="J5" s="103"/>
+      <c r="K5" s="103"/>
       <c r="L5" s="39" t="s">
         <v>17</v>
       </c>
@@ -5626,7 +5616,7 @@
       </c>
       <c r="N5" s="39"/>
       <c r="O5" s="43"/>
-      <c r="P5" s="104"/>
+      <c r="P5" s="101"/>
     </row>
     <row r="6" spans="1:16" ht="30">
       <c r="A6" s="6" t="s">
@@ -6143,11 +6133,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A4:A5"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="C4:C5"/>
-    <mergeCell ref="D4:D5"/>
-    <mergeCell ref="E4:E5"/>
     <mergeCell ref="K4:K5"/>
     <mergeCell ref="P4:P5"/>
     <mergeCell ref="G2:L3"/>
@@ -6156,6 +6141,11 @@
     <mergeCell ref="H4:H5"/>
     <mergeCell ref="I4:I5"/>
     <mergeCell ref="J4:J5"/>
+    <mergeCell ref="A4:A5"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="D4:D5"/>
+    <mergeCell ref="E4:E5"/>
   </mergeCells>
   <conditionalFormatting sqref="K6:K17">
     <cfRule type="containsText" dxfId="35" priority="1" operator="containsText" text="REGISTERED">
@@ -6217,7 +6207,7 @@
     <row r="2" spans="1:16" ht="21" customHeight="1">
       <c r="A2" s="18">
         <f ca="1">TODAY()</f>
-        <v>46083</v>
+        <v>46085</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="14.45" customHeight="1">
@@ -6240,34 +6230,34 @@
       <c r="A5" s="93" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="104" t="s">
+      <c r="B5" s="101" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="104" t="s">
+      <c r="C5" s="101" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="104" t="s">
+      <c r="D5" s="101" t="s">
         <v>5</v>
       </c>
-      <c r="E5" s="104" t="s">
+      <c r="E5" s="101" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="104" t="s">
+      <c r="F5" s="101" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="104" t="s">
+      <c r="G5" s="101" t="s">
         <v>8</v>
       </c>
-      <c r="H5" s="104" t="s">
+      <c r="H5" s="101" t="s">
         <v>9</v>
       </c>
-      <c r="I5" s="104" t="s">
+      <c r="I5" s="101" t="s">
         <v>10</v>
       </c>
-      <c r="J5" s="104" t="s">
+      <c r="J5" s="101" t="s">
         <v>11</v>
       </c>
-      <c r="K5" s="103" t="s">
+      <c r="K5" s="104" t="s">
         <v>148</v>
       </c>
       <c r="L5" s="108" t="s">
@@ -6286,16 +6276,16 @@
     </row>
     <row r="6" spans="1:16">
       <c r="A6" s="100"/>
-      <c r="B6" s="104"/>
-      <c r="C6" s="104"/>
-      <c r="D6" s="104"/>
-      <c r="E6" s="104"/>
-      <c r="F6" s="104"/>
-      <c r="G6" s="104"/>
-      <c r="H6" s="104"/>
-      <c r="I6" s="104"/>
-      <c r="J6" s="104"/>
-      <c r="K6" s="103"/>
+      <c r="B6" s="101"/>
+      <c r="C6" s="101"/>
+      <c r="D6" s="101"/>
+      <c r="E6" s="101"/>
+      <c r="F6" s="101"/>
+      <c r="G6" s="101"/>
+      <c r="H6" s="101"/>
+      <c r="I6" s="101"/>
+      <c r="J6" s="101"/>
+      <c r="K6" s="104"/>
       <c r="L6" s="39" t="s">
         <v>17</v>
       </c>
@@ -6738,7 +6728,7 @@
     <row r="2" spans="1:16" ht="14.45" customHeight="1">
       <c r="A2" s="18">
         <f ca="1">TODAY()</f>
-        <v>46083</v>
+        <v>46085</v>
       </c>
       <c r="F2" s="98" t="s">
         <v>1</v>
@@ -8421,7 +8411,7 @@
     <row r="2" spans="1:16" ht="14.45" customHeight="1">
       <c r="A2" s="18">
         <f ca="1">TODAY()</f>
-        <v>46083</v>
+        <v>46085</v>
       </c>
       <c r="F2" s="98"/>
       <c r="G2" s="98"/>
@@ -9186,7 +9176,7 @@
     <row r="2" spans="1:16" ht="14.45" customHeight="1">
       <c r="A2" s="4">
         <f ca="1">TODAY()</f>
-        <v>46083</v>
+        <v>46085</v>
       </c>
       <c r="F2" s="98" t="s">
         <v>1</v>

</xml_diff>